<commit_message>
actualización gráficos y última versión de la base de datos
</commit_message>
<xml_diff>
--- a/input/260427-diccionario.xlsx
+++ b/input/260427-diccionario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soledadaraya/Library/CloudStorage/Dropbox/Lucía Miranda Fondecyt/femocratas/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCBEE660-F2DC-E941-9C74-A1BF373CB0BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D0B3F6-9191-4943-B095-B21530CCFD70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2220" yWindow="3800" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4752" uniqueCount="3602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4753" uniqueCount="3603">
   <si>
     <t>tokens</t>
   </si>
@@ -10829,6 +10829,9 @@
   </si>
   <si>
     <t>mov_feminista</t>
+  </si>
+  <si>
+    <t>en_el_fondo</t>
   </si>
 </sst>
 </file>
@@ -11247,7 +11250,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M3592"/>
+  <dimension ref="A1:M3593"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -11375,6 +11378,9 @@
       <c r="B7">
         <v>9</v>
       </c>
+      <c r="C7" s="3">
+        <v>1</v>
+      </c>
       <c r="G7">
         <v>1</v>
       </c>
@@ -11397,6 +11403,9 @@
       <c r="B9">
         <v>8</v>
       </c>
+      <c r="C9" s="3">
+        <v>1</v>
+      </c>
       <c r="G9">
         <v>1</v>
       </c>
@@ -11408,6 +11417,9 @@
       <c r="B10">
         <v>5</v>
       </c>
+      <c r="C10" s="3">
+        <v>1</v>
+      </c>
       <c r="G10">
         <v>1</v>
       </c>
@@ -11419,6 +11431,9 @@
       <c r="B11">
         <v>15</v>
       </c>
+      <c r="C11" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -11427,6 +11442,9 @@
       <c r="B12">
         <v>5</v>
       </c>
+      <c r="C12" s="3">
+        <v>1</v>
+      </c>
       <c r="G12">
         <v>1</v>
       </c>
@@ -26773,9 +26791,6 @@
       <c r="B1406">
         <v>137</v>
       </c>
-      <c r="C1406" s="3">
-        <v>1</v>
-      </c>
       <c r="E1406">
         <v>1</v>
       </c>
@@ -27791,6 +27806,9 @@
       <c r="E1501">
         <v>1</v>
       </c>
+      <c r="H1501" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="1502" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1502" t="s">
@@ -37553,6 +37571,9 @@
       <c r="G2380">
         <v>1</v>
       </c>
+      <c r="H2380" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="2381" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2381" t="s">
@@ -37564,6 +37585,9 @@
       <c r="G2381">
         <v>1</v>
       </c>
+      <c r="H2381" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="2382" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2382" t="s">
@@ -37575,6 +37599,9 @@
       <c r="G2382">
         <v>1</v>
       </c>
+      <c r="H2382" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="2383" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2383" t="s">
@@ -37583,6 +37610,9 @@
       <c r="B2383">
         <v>10</v>
       </c>
+      <c r="H2383" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="2384" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2384" t="s">
@@ -51241,6 +51271,14 @@
       </c>
       <c r="B3592">
         <v>10</v>
+      </c>
+    </row>
+    <row r="3593" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3593" t="s">
+        <v>3602</v>
+      </c>
+      <c r="C3593" s="3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>